<commit_message>
CoQ register: the IJZ-MB delivery of 25/26.08.2026 is campaign sampling for every lot
The 30 microbiology samples reached the laboratory on 25 and 26.08.2026
under consecutive requests 295–324/2026, 68 to 436 days after packaging,
against the one to two weeks release testing takes; the release testing
of the four post-SOP lots among them is their CNP certificate of 30.06 or
06.07.2026. So every certificate of that delivery is a retest document,
whatever the lot's group (--campaign-manifest=, the split manifest). The
four CoQs move from 07.09.2026 back to their CNP-based rule dates with
#9 named as the initial certificate to locate (IJZ).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_gap_analysis/tracker/Issuance_Registers_prelim.xlsx
+++ b/deliverables/qc_gap_analysis/tracker/Issuance_Registers_prelim.xlsx
@@ -12971,7 +12971,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>retest — not yet sampled</t>
+          <t>retest — sampled — Tranche 2/3 (potency and mycotoxins pending)</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -13053,7 +13053,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>retest — not yet sampled</t>
+          <t>retest — sampled — Tranche 2/3 (potency and mycotoxins pending)</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -13217,7 +13217,7 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>retest — not yet sampled</t>
+          <t>retest — sampled — Tranche 2/3 (potency and mycotoxins pending)</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
@@ -13954,7 +13954,7 @@
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -14050,7 +14050,7 @@
       </c>
       <c r="T6" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -14146,7 +14146,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -15558,7 +15558,7 @@
       </c>
       <c r="T22" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -17906,7 +17906,7 @@
       </c>
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18000,7 +18000,7 @@
       </c>
       <c r="T48" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18094,7 +18094,7 @@
       </c>
       <c r="T49" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18188,7 +18188,7 @@
       </c>
       <c r="T50" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18282,7 +18282,7 @@
       </c>
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18376,7 +18376,7 @@
       </c>
       <c r="T52" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18470,7 +18470,7 @@
       </c>
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18564,7 +18564,7 @@
       </c>
       <c r="T54" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18846,7 +18846,7 @@
       </c>
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -18940,7 +18940,7 @@
       </c>
       <c r="T58" s="7" t="inlineStr">
         <is>
-          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — legacy series, issued 27.05.2026 · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -19784,7 +19784,7 @@
       </c>
       <c r="T67" s="7" t="inlineStr">
         <is>
-          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -19974,7 +19974,7 @@
       </c>
       <c r="T69" s="7" t="inlineStr">
         <is>
-          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20011,11 +20011,11 @@
         </is>
       </c>
       <c r="H70" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060382|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060342|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I70" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060382|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060342|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -20030,12 +20030,12 @@
       </c>
       <c r="L70" s="3" t="inlineStr">
         <is>
-          <t>SCR012603</t>
+          <t>SCR012601* (from the list)</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>P060382</t>
+          <t>P060342</t>
         </is>
       </c>
       <c r="N70" s="2" t="inlineStr">
@@ -20060,17 +20060,17 @@
       </c>
       <c r="R70" s="2" t="inlineStr">
         <is>
-          <t>CoQ-PP-2026-0026</t>
+          <t>— not in the issuance plan —</t>
         </is>
       </c>
       <c r="S70" s="2" t="inlineStr">
         <is>
-          <t>P060382|I</t>
+          <t>P060342|I</t>
         </is>
       </c>
       <c r="T70" s="7" t="inlineStr">
         <is>
-          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #9, #10, #11, #12</t>
+          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20096,20 +20096,22 @@
         <f>IF(ISNUMBER(F71),IF(AND(J71="legacy",F71&lt;=DATE(2026,5,27)),DATE(2026,5,27),MAX(DATE(2026,5,27),(F71+7)+CHOOSE(WEEKDAY(F71+7,2),0,0,0,0,0,2,1))),IF(J71="legacy",DATE(2026,5,27),""))</f>
         <v/>
       </c>
-      <c r="F71" s="5" t="n">
-        <v>46203</v>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>ППК26111</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H71" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060362|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060382|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I71" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060362|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060382|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -20124,23 +20126,27 @@
       </c>
       <c r="L71" s="3" t="inlineStr">
         <is>
-          <t>JD012603</t>
+          <t>SCR012603</t>
         </is>
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>P060362</t>
-        </is>
-      </c>
-      <c r="N71" s="2" t="inlineStr"/>
-      <c r="O71" s="2" t="inlineStr">
-        <is>
-          <t>ППК26111, (30.06.2026) [CNP]</t>
-        </is>
-      </c>
-      <c r="P71" s="2" t="inlineStr">
-        <is>
-          <t>A: ППК26111 / B: ППК26111 / FM: ППК26111</t>
+          <t>P060382</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>Scrambler</t>
+        </is>
+      </c>
+      <c r="O71" s="6" t="inlineStr">
+        <is>
+          <t>— no cannabinoid certificate from the initial testing —</t>
+        </is>
+      </c>
+      <c r="P71" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="Q71" s="2" t="inlineStr">
@@ -20150,17 +20156,17 @@
       </c>
       <c r="R71" s="2" t="inlineStr">
         <is>
-          <t>CoQ-PP-2026-0020</t>
+          <t>CoQ-PP-2026-0026</t>
         </is>
       </c>
       <c r="S71" s="2" t="inlineStr">
         <is>
-          <t>P060362|I</t>
+          <t>P060382|I</t>
         </is>
       </c>
       <c r="T71" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — provisional date: no initial certificate on file yet — the date follows the latest eCoA once located · initial certificate to locate: #3 (CNP), #4 (CNP), #5 (CNP), #6 (CNP), #8 (CNP), #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20191,15 +20197,15 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>ППК26111</t>
+          <t>ППК26110</t>
         </is>
       </c>
       <c r="H72" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060422|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060392|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I72" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060422|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060392|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -20214,23 +20220,27 @@
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>JD012603</t>
+          <t>FB012603V</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>P060422</t>
-        </is>
-      </c>
-      <c r="N72" s="2" t="inlineStr"/>
+          <t>P060392</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Fat Bastard</t>
+        </is>
+      </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ППК26111, (30.06.2026) [CNP]</t>
+          <t>ППК26110, (30.06.2026) [CNP]</t>
         </is>
       </c>
       <c r="P72" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26111 / B: ППК26111 / FM: ППК26111</t>
+          <t>A: ППК26110 / B: ППК26110 / FM: ППК26110</t>
         </is>
       </c>
       <c r="Q72" s="2" t="inlineStr">
@@ -20240,17 +20250,17 @@
       </c>
       <c r="R72" s="2" t="inlineStr">
         <is>
-          <t>CoQ-PP-2026-0022</t>
+          <t>(assigned on issue)</t>
         </is>
       </c>
       <c r="S72" s="2" t="inlineStr">
         <is>
-          <t>P060422|I</t>
+          <t>P060392|I</t>
         </is>
       </c>
       <c r="T72" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20281,15 +20291,15 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>ППК26114</t>
+          <t>ППК26111</t>
         </is>
       </c>
       <c r="H73" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060402|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060362|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I73" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060402|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060362|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -20304,27 +20314,23 @@
       </c>
       <c r="L73" s="3" t="inlineStr">
         <is>
-          <t>GG012603</t>
+          <t>JD012603</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>P060402</t>
-        </is>
-      </c>
-      <c r="N73" s="2" t="inlineStr">
-        <is>
-          <t>GorillaGlue</t>
-        </is>
-      </c>
+          <t>P060362</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr"/>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ППК26114, (30.06.2026) [CNP]</t>
+          <t>ППК26111, (30.06.2026) [CNP]</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26114 / B: ППК26114 / FM: ППК26114</t>
+          <t>A: ППК26111 / B: ППК26111 / FM: ППК26111</t>
         </is>
       </c>
       <c r="Q73" s="2" t="inlineStr">
@@ -20334,17 +20340,17 @@
       </c>
       <c r="R73" s="2" t="inlineStr">
         <is>
-          <t>CoQ-PP-2026-0023</t>
+          <t>CoQ-PP-2026-0020</t>
         </is>
       </c>
       <c r="S73" s="2" t="inlineStr">
         <is>
-          <t>P060402|I</t>
+          <t>P060362|I</t>
         </is>
       </c>
       <c r="T73" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20379,11 +20385,11 @@
         </is>
       </c>
       <c r="H74" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060412|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060422|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I74" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060412|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060422|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -20403,7 +20409,7 @@
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>P060412</t>
+          <t>P060422</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr"/>
@@ -20424,17 +20430,17 @@
       </c>
       <c r="R74" s="2" t="inlineStr">
         <is>
-          <t>CoQ-PP-2026-0025</t>
+          <t>CoQ-PP-2026-0022</t>
         </is>
       </c>
       <c r="S74" s="2" t="inlineStr">
         <is>
-          <t>P060412|I</t>
+          <t>P060422|I</t>
         </is>
       </c>
       <c r="T74" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20461,19 +20467,19 @@
         <v/>
       </c>
       <c r="F75" s="5" t="n">
-        <v>46224</v>
+        <v>46203</v>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>ППК26127</t>
+          <t>ППК26114</t>
         </is>
       </c>
       <c r="H75" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060452|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060402|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I75" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060452|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060402|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -20488,27 +20494,27 @@
       </c>
       <c r="L75" s="3" t="inlineStr">
         <is>
-          <t>FB032601</t>
+          <t>GG012603</t>
         </is>
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>P060452</t>
+          <t>P060402</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>FatBastard</t>
+          <t>GorillaGlue</t>
         </is>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ППК26127, (21.07.2026) [CNP]</t>
+          <t>ППК26114, (30.06.2026) [CNP]</t>
         </is>
       </c>
       <c r="P75" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26127 / B: ППК26127 / FM: ППК26127</t>
+          <t>A: ППК26114 / B: ППК26114 / FM: ППК26114</t>
         </is>
       </c>
       <c r="Q75" s="2" t="inlineStr">
@@ -20518,17 +20524,17 @@
       </c>
       <c r="R75" s="2" t="inlineStr">
         <is>
-          <t>(assigned on issue)</t>
+          <t>CoQ-PP-2026-0023</t>
         </is>
       </c>
       <c r="S75" s="2" t="inlineStr">
         <is>
-          <t>P060452|I</t>
+          <t>P060402|I</t>
         </is>
       </c>
       <c r="T75" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20555,19 +20561,19 @@
         <v/>
       </c>
       <c r="F76" s="5" t="n">
-        <v>46224</v>
+        <v>46203</v>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>ППК26128</t>
+          <t>ППК26111</t>
         </is>
       </c>
       <c r="H76" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060462|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060412|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I76" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060462|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060412|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -20582,27 +20588,23 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>GG032601</t>
+          <t>JD012603</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>P060462</t>
-        </is>
-      </c>
-      <c r="N76" s="2" t="inlineStr">
-        <is>
-          <t>GorillaGlue</t>
-        </is>
-      </c>
+          <t>P060412</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr"/>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ППК26128, (21.07.2026) [CNP]</t>
+          <t>ППК26111, (30.06.2026) [CNP]</t>
         </is>
       </c>
       <c r="P76" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26128 / B: ППК26128 / FM: ППК26128</t>
+          <t>A: ППК26111 / B: ППК26111 / FM: ППК26111</t>
         </is>
       </c>
       <c r="Q76" s="2" t="inlineStr">
@@ -20612,17 +20614,17 @@
       </c>
       <c r="R76" s="2" t="inlineStr">
         <is>
-          <t>(assigned on issue)</t>
+          <t>CoQ-PP-2026-0025</t>
         </is>
       </c>
       <c r="S76" s="2" t="inlineStr">
         <is>
-          <t>P060462|I</t>
+          <t>P060412|I</t>
         </is>
       </c>
       <c r="T76" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20653,15 +20655,15 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>ППК26115</t>
+          <t>ППК26112</t>
         </is>
       </c>
       <c r="H77" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060482|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060432|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I77" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060482|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060432|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -20676,27 +20678,27 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>JD022601</t>
+          <t>FB012603</t>
         </is>
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>P060482</t>
+          <t>P060432</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>JellyDonutz</t>
+          <t>Fat Bastard</t>
         </is>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ППК26115, (30.06.2026) [CNP]</t>
+          <t>ППК26112, (30.06.2026) [CNP]</t>
         </is>
       </c>
       <c r="P77" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26115 / B: ППК26115 / FM: ППК26115</t>
+          <t>A: ППК26112 / B: ППК26112 / FM: ППК26112</t>
         </is>
       </c>
       <c r="Q77" s="2" t="inlineStr">
@@ -20711,12 +20713,12 @@
       </c>
       <c r="S77" s="2" t="inlineStr">
         <is>
-          <t>P060482|I</t>
+          <t>P060432|I</t>
         </is>
       </c>
       <c r="T77" s="7" t="inlineStr">
         <is>
-          <t>registered — held to the packaging date · initial certificate to locate (CNP): #9, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20743,19 +20745,19 @@
         <v/>
       </c>
       <c r="F78" s="5" t="n">
-        <v>46265</v>
+        <v>46209</v>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>538-1069-26</t>
+          <t>ППК26116</t>
         </is>
       </c>
       <c r="H78" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060392|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060442|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I78" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060392|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060442|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -20770,27 +20772,27 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>FB012603V</t>
+          <t>SCR022601</t>
         </is>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>P060392</t>
+          <t>P060442</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>Fat Bastard</t>
+          <t>Scrambler</t>
         </is>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ППК26110, (30.06.2026) [CNP]</t>
+          <t>ППК26116, (06.07.2026) [CNP]</t>
         </is>
       </c>
       <c r="P78" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26110 / B: ППК26110 / FM: ППК26110</t>
+          <t>A: ППК26116 / B: ППК26116 / FM: ППК26116</t>
         </is>
       </c>
       <c r="Q78" s="2" t="inlineStr">
@@ -20805,12 +20807,12 @@
       </c>
       <c r="S78" s="2" t="inlineStr">
         <is>
-          <t>P060392|I</t>
+          <t>P060442|I</t>
         </is>
       </c>
       <c r="T78" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20837,19 +20839,19 @@
         <v/>
       </c>
       <c r="F79" s="5" t="n">
-        <v>46265</v>
+        <v>46224</v>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>539-1070-26</t>
+          <t>ППК26127</t>
         </is>
       </c>
       <c r="H79" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060342|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060452|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I79" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060342|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060452|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -20864,27 +20866,27 @@
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>SCR012601* (from the list)</t>
+          <t>FB032601</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>P060342</t>
+          <t>P060452</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>Scrambler</t>
-        </is>
-      </c>
-      <c r="O79" s="6" t="inlineStr">
-        <is>
-          <t>— no cannabinoid certificate from the initial testing —</t>
-        </is>
-      </c>
-      <c r="P79" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>FatBastard</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>ППК26127, (21.07.2026) [CNP]</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>A: ППК26127 / B: ППК26127 / FM: ППК26127</t>
         </is>
       </c>
       <c r="Q79" s="2" t="inlineStr">
@@ -20894,17 +20896,17 @@
       </c>
       <c r="R79" s="2" t="inlineStr">
         <is>
-          <t>— not in the issuance plan —</t>
+          <t>(assigned on issue)</t>
         </is>
       </c>
       <c r="S79" s="2" t="inlineStr">
         <is>
-          <t>P060342|I</t>
+          <t>P060452|I</t>
         </is>
       </c>
       <c r="T79" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #3, #4, #5, #6, #8, #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -20931,19 +20933,19 @@
         <v/>
       </c>
       <c r="F80" s="5" t="n">
-        <v>46265</v>
+        <v>46224</v>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>537-1068-26</t>
+          <t>ППК26128</t>
         </is>
       </c>
       <c r="H80" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060432|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060462|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I80" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060432|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060462|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -20958,27 +20960,27 @@
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>FB012603</t>
+          <t>GG032601</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>P060432</t>
+          <t>P060462</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>Fat Bastard</t>
+          <t>GorillaGlue</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ППК26112, (30.06.2026) [CNP]</t>
+          <t>ППК26128, (21.07.2026) [CNP]</t>
         </is>
       </c>
       <c r="P80" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26112 / B: ППК26112 / FM: ППК26112</t>
+          <t>A: ППК26128 / B: ППК26128 / FM: ППК26128</t>
         </is>
       </c>
       <c r="Q80" s="2" t="inlineStr">
@@ -20993,12 +20995,12 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
-          <t>P060432|I</t>
+          <t>P060462|I</t>
         </is>
       </c>
       <c r="T80" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #10, #11, #12</t>
+          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -21025,19 +21027,19 @@
         <v/>
       </c>
       <c r="F81" s="5" t="n">
-        <v>46265</v>
+        <v>46203</v>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>536-1067-26</t>
+          <t>ППК26115</t>
         </is>
       </c>
       <c r="H81" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060442|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P060482|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I81" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060442|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P060482|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -21052,27 +21054,27 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>SCR022601</t>
+          <t>JD022601</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>P060442</t>
+          <t>P060482</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>Scrambler</t>
+          <t>JellyDonutz</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ППК26116, (06.07.2026) [CNP]</t>
+          <t>ППК26115, (30.06.2026) [CNP]</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
         <is>
-          <t>A: ППК26116 / B: ППК26116 / FM: ППК26116</t>
+          <t>A: ППК26115 / B: ППК26115 / FM: ППК26115</t>
         </is>
       </c>
       <c r="Q81" s="2" t="inlineStr">
@@ -21087,12 +21089,12 @@
       </c>
       <c r="S81" s="2" t="inlineStr">
         <is>
-          <t>P060442|I</t>
+          <t>P060482|I</t>
         </is>
       </c>
       <c r="T81" s="7" t="inlineStr">
         <is>
-          <t>registered — first working day 7 days after the latest eCoA · initial certificate to locate (CNP): #10, #11, #12</t>
+          <t>registered — held to the packaging date · initial certificate to locate: #9 (IJZ), #10 (CNP), #11 (CNP), #12 (CNP)</t>
         </is>
       </c>
     </row>
@@ -27808,14 +27810,12 @@
         <f>IF(ISNUMBER(F153),MAX(DATE(2026,5,27),(F153+7)+CHOOSE(WEEKDAY(F153+7,2),0,0,0,0,0,2,1)),"at retest sampling")</f>
         <v/>
       </c>
-      <c r="F153" s="5" t="inlineStr">
-        <is>
-          <t>— not yet sampled —</t>
-        </is>
+      <c r="F153" s="5" t="n">
+        <v>46265</v>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>537-1068-26</t>
         </is>
       </c>
       <c r="H153" s="2">
@@ -27833,7 +27833,7 @@
       </c>
       <c r="K153" s="2" t="inlineStr">
         <is>
-          <t>retest — not yet sampled</t>
+          <t>retest — sampled — Tranche 2/3 (potency and mycotoxins pending)</t>
         </is>
       </c>
       <c r="L153" s="3" t="inlineStr">
@@ -27878,7 +27878,7 @@
       </c>
       <c r="T153" s="9" t="inlineStr">
         <is>
-          <t>not yet issuable — pending — not yet sampled · issued on the first working day 7 days after the latest retest certificate, once the in-house iCoA exists</t>
+          <t>not yet issuable — sampled — microbiology on file, retest assay pending · issued on the first working day 7 days after the latest retest certificate, once the in-house iCoA exists</t>
         </is>
       </c>
     </row>
@@ -27904,14 +27904,12 @@
         <f>IF(ISNUMBER(F154),MAX(DATE(2026,5,27),(F154+7)+CHOOSE(WEEKDAY(F154+7,2),0,0,0,0,0,2,1)),"at retest sampling")</f>
         <v/>
       </c>
-      <c r="F154" s="5" t="inlineStr">
-        <is>
-          <t>— not yet sampled —</t>
-        </is>
+      <c r="F154" s="5" t="n">
+        <v>46265</v>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>538-1069-26</t>
         </is>
       </c>
       <c r="H154" s="2">
@@ -27929,7 +27927,7 @@
       </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
-          <t>retest — not yet sampled</t>
+          <t>retest — sampled — Tranche 2/3 (potency and mycotoxins pending)</t>
         </is>
       </c>
       <c r="L154" s="3" t="inlineStr">
@@ -27974,7 +27972,7 @@
       </c>
       <c r="T154" s="9" t="inlineStr">
         <is>
-          <t>not yet issuable — pending — not yet sampled · issued on the first working day 7 days after the latest retest certificate, once the in-house iCoA exists</t>
+          <t>not yet issuable — sampled — microbiology on file, retest assay pending · issued on the first working day 7 days after the latest retest certificate, once the in-house iCoA exists</t>
         </is>
       </c>
     </row>
@@ -28096,14 +28094,12 @@
         <f>IF(ISNUMBER(F156),MAX(DATE(2026,5,27),(F156+7)+CHOOSE(WEEKDAY(F156+7,2),0,0,0,0,0,2,1)),"at retest sampling")</f>
         <v/>
       </c>
-      <c r="F156" s="5" t="inlineStr">
-        <is>
-          <t>— not yet sampled —</t>
-        </is>
+      <c r="F156" s="5" t="n">
+        <v>46265</v>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>536-1067-26</t>
         </is>
       </c>
       <c r="H156" s="2">
@@ -28121,7 +28117,7 @@
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>retest — not yet sampled</t>
+          <t>retest — sampled — Tranche 2/3 (potency and mycotoxins pending)</t>
         </is>
       </c>
       <c r="L156" s="3" t="inlineStr">
@@ -28166,7 +28162,7 @@
       </c>
       <c r="T156" s="9" t="inlineStr">
         <is>
-          <t>not yet issuable — pending — not yet sampled · issued on the first working day 7 days after the latest retest certificate, once the in-house iCoA exists</t>
+          <t>not yet issuable — sampled — microbiology on file, retest assay pending · issued on the first working day 7 days after the latest retest certificate, once the in-house iCoA exists</t>
         </is>
       </c>
     </row>
@@ -28365,7 +28361,7 @@
     <row r="160" ht="150" customHeight="1">
       <c r="A160" s="10" t="inlineStr">
         <is>
-          <t>Head of QC, 05.09.2026: preliminary CoQ issuance register — codes CoQ-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, in the order of issue. LEGACY lots (packed before the SOP floor of 11.05.2026, or holding an old in-house QCCoA 001 certificate, which the CoQ supersedes) are all issued on 27.05.2026, in chronological order of packaging; POST-SOP lots follow, each on the first working day 7 days after the latest eCoA the CoQ cites and never before 27.05.2026, so the legacy series keeps 001 onward. Every CoQ cites its lot's iCoA (identification A, B, foreign matter) and reports identification C as 'Conforms', referenced to the eCoA that covers Total THC. ADHERENCE (ISSUE_COQ_CONVENTIONS): a CoQ never precedes a document it cites — a legacy lot whose latest eCoA is dated after 27.05.2026 takes the post-SOP rule and is flagged in Status; a CoQ never precedes its iCoA; Head of QC, 05.09.2026 (evening): a production lot whose initial certificate for a determination is not on file keeps its planned CoQ and number — the initial testing exists at the Faculty of Pharmacy's Center for Natural Products and the certificate is to be located (Work Order; Status names the determination); a certificate dated on or after 01.07.2026 is a retest document (the QP's campaign: Tranche 1, the first 21 lots, sampled July 2026; then Tranches 2 and 3) and never certifies the initial CoQ — a determination whose only certificate is a retest one is uncertified for the legacy CoQ and flagged; nothing is dated on a weekend. RETEST ROWS: the reissued CoQ carries the retest results (cannabinoids with identification C by Farmahem, mycotoxins, microbiology by IJZ-MB) and the initial certificates for the rest; its rule date is the first working day 7 days after the latest retest certificate, and it is issued once the in-house retest iCoA exists. FORMULAS: No. and the code as on the iCoA Register; Rule date is 27.05.2026 for a legacy row whose latest eCoA is on or before it, else the first working day 7 days after the latest eCoA (not before 27.05.2026); the planned date is the latest of the rule date, the iCoA's date and the lot's last day of packaging; iCoA (register) and its date are looked up on the iCoA Register by Key. The latest eCoA cited is a value (the first credited certificate per determination dated before the retest campaign; for a retest row, the latest retest certificate), recomputed by the builder. Working days are Monday to Friday; public holidays are not applied. FLAGS: P060272: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060322: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060292: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060302: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060402: no initial certificate for #10 — only the retest 197-8-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060142: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060182: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | HPA1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-13-K-26 of 07.08.2026 / 197-13-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060152: no initial certificate for #10 — only the retest 197-16-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060202: no initial certificate for #9 — only the retest 547-1078-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060262: post-SOP CoQ rule date 30.04.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060312: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060482: CoQ rule date 07.07.2026 precedes the packaging of the lot (05.08.2026) — held to the packaging date | OPM1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-17-K-26 of 07.08.2026 / 197-17-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060222: no initial certificate for #9 — only the retest 546-1077-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060332: no initial certificate on file — the CoQ keeps its planned number with a provisional date 27.05.2026 | P060332: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-6-K-26 of 07.08.2026 / 197-6-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060352: no initial certificate on file — the CoQ keeps its planned number with a provisional date 28.05.2026 | P060352: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-7-K-26 of 07.08.2026 / 197-7-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060382: no initial certificate on file — the CoQ keeps its planned number with a provisional date 01.06.2026 | P060382: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-21-K-26 of 07.08.2026 / 197-21-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060282: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060162: no initial certificate for #9 — only the retest 549-1080-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P050142: no initial certificate for #9 — only the retest 559-1090-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060102: no initial certificate for #9 — only the retest 551-1082-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue)</t>
+          <t>Head of QC, 05.09.2026: preliminary CoQ issuance register — codes CoQ-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, in the order of issue. LEGACY lots (packed before the SOP floor of 11.05.2026, or holding an old in-house QCCoA 001 certificate, which the CoQ supersedes) are all issued on 27.05.2026, in chronological order of packaging; POST-SOP lots follow, each on the first working day 7 days after the latest eCoA the CoQ cites and never before 27.05.2026, so the legacy series keeps 001 onward. Every CoQ cites its lot's iCoA (identification A, B, foreign matter) and reports identification C as 'Conforms', referenced to the eCoA that covers Total THC. ADHERENCE (ISSUE_COQ_CONVENTIONS): a CoQ never precedes a document it cites — a legacy lot whose latest eCoA is dated after 27.05.2026 takes the post-SOP rule and is flagged in Status; a CoQ never precedes its iCoA; Head of QC, 05.09.2026 (evening): a production lot whose initial certificate for a determination is not on file keeps its planned CoQ and number — the initial testing exists at the Faculty of Pharmacy's Center for Natural Products (microbiology: IJZ) and the certificate is to be located (Work Order; Status names the determination); a certificate dated on or after 01.07.2026 is a retest document (the QP's campaign: Tranche 1, the first 21 lots, sampled July 2026; then Tranches 2 and 3) and never certifies the initial CoQ — a determination whose only certificate is a retest one is uncertified for the legacy CoQ and flagged; the IJZ-MB delivery of 25/26.08.2026 (certificates of 31.08 and 01.09.2026, 68 to 436 days after packaging) is one campaign sampling and every certificate in it is a retest document, for the post-SOP lots too; nothing is dated on a weekend. RETEST ROWS: the reissued CoQ carries the retest results (cannabinoids with identification C by Farmahem, mycotoxins, microbiology by IJZ-MB) and the initial certificates for the rest; its rule date is the first working day 7 days after the latest retest certificate, and it is issued once the in-house retest iCoA exists. FORMULAS: No. and the code as on the iCoA Register; Rule date is 27.05.2026 for a legacy row whose latest eCoA is on or before it, else the first working day 7 days after the latest eCoA (not before 27.05.2026); the planned date is the latest of the rule date, the iCoA's date and the lot's last day of packaging; iCoA (register) and its date are looked up on the iCoA Register by Key. The latest eCoA cited is a value (the first credited certificate per determination dated before the retest campaign; for a retest row, the latest retest certificate), recomputed by the builder. Working days are Monday to Friday; public holidays are not applied. FLAGS: P060272: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060322: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060432: no initial certificate for #9 — only the retest 537-1068-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060392: no initial certificate for #9 — only the retest 538-1069-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060292: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060302: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060402: no initial certificate for #10 — only the retest 197-8-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060142: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060182: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | HPA1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-13-K-26 of 07.08.2026 / 197-13-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060152: no initial certificate for #10 — only the retest 197-16-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060202: no initial certificate for #9 — only the retest 547-1078-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060262: post-SOP CoQ rule date 30.04.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060312: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060482: CoQ rule date 07.07.2026 precedes the packaging of the lot (05.08.2026) — held to the packaging date | OPM1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-17-K-26 of 07.08.2026 / 197-17-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060222: no initial certificate for #9 — only the retest 546-1077-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060332: no initial certificate on file — the CoQ keeps its planned number with a provisional date 27.05.2026 | P060332: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-6-K-26 of 07.08.2026 / 197-6-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060352: no initial certificate on file — the CoQ keeps its planned number with a provisional date 28.05.2026 | P060352: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-7-K-26 of 07.08.2026 / 197-7-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060382: no initial certificate on file — the CoQ keeps its planned number with a provisional date 01.06.2026 | P060382: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-21-K-26 of 07.08.2026 / 197-21-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060442: no initial certificate for #9 — only the retest 536-1067-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060282: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060162: no initial certificate for #9 — only the retest 549-1080-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P050142: no initial certificate for #9 — only the retest 559-1090-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060102: no initial certificate for #9 — only the retest 551-1082-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060342: no initial certificate on file — the CoQ keeps its planned number with a provisional date 01.06.2026 | P060342: no initial certificate for #9 — only the retest 539-1070-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue)</t>
         </is>
       </c>
     </row>
@@ -31750,7 +31746,7 @@
     <row r="3" ht="190" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Head of QC, 05.09.2026: preliminary CoQ issuance register — codes CoQ-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, in the order of issue. LEGACY lots (packed before the SOP floor of 11.05.2026, or holding an old in-house QCCoA 001 certificate, which the CoQ supersedes) are all issued on 27.05.2026, in chronological order of packaging; POST-SOP lots follow, each on the first working day 7 days after the latest eCoA the CoQ cites and never before 27.05.2026, so the legacy series keeps 001 onward. Every CoQ cites its lot's iCoA (identification A, B, foreign matter) and reports identification C as 'Conforms', referenced to the eCoA that covers Total THC. ADHERENCE (ISSUE_COQ_CONVENTIONS): a CoQ never precedes a document it cites — a legacy lot whose latest eCoA is dated after 27.05.2026 takes the post-SOP rule and is flagged in Status; a CoQ never precedes its iCoA; Head of QC, 05.09.2026 (evening): a production lot whose initial certificate for a determination is not on file keeps its planned CoQ and number — the initial testing exists at the Faculty of Pharmacy's Center for Natural Products and the certificate is to be located (Work Order; Status names the determination); a certificate dated on or after 01.07.2026 is a retest document (the QP's campaign: Tranche 1, the first 21 lots, sampled July 2026; then Tranches 2 and 3) and never certifies the initial CoQ — a determination whose only certificate is a retest one is uncertified for the legacy CoQ and flagged; nothing is dated on a weekend. RETEST ROWS: the reissued CoQ carries the retest results (cannabinoids with identification C by Farmahem, mycotoxins, microbiology by IJZ-MB) and the initial certificates for the rest; its rule date is the first working day 7 days after the latest retest certificate, and it is issued once the in-house retest iCoA exists. FORMULAS: No. and the code as on the iCoA Register; Rule date is 27.05.2026 for a legacy row whose latest eCoA is on or before it, else the first working day 7 days after the latest eCoA (not before 27.05.2026); the planned date is the latest of the rule date, the iCoA's date and the lot's last day of packaging; iCoA (register) and its date are looked up on the iCoA Register by Key. The latest eCoA cited is a value (the first credited certificate per determination dated before the retest campaign; for a retest row, the latest retest certificate), recomputed by the builder. Working days are Monday to Friday; public holidays are not applied. FLAGS: P060272: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060322: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060292: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060302: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060402: no initial certificate for #10 — only the retest 197-8-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060142: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060182: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | HPA1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-13-K-26 of 07.08.2026 / 197-13-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060152: no initial certificate for #10 — only the retest 197-16-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060202: no initial certificate for #9 — only the retest 547-1078-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060262: post-SOP CoQ rule date 30.04.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060312: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060482: CoQ rule date 07.07.2026 precedes the packaging of the lot (05.08.2026) — held to the packaging date | OPM1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-17-K-26 of 07.08.2026 / 197-17-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060222: no initial certificate for #9 — only the retest 546-1077-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060332: no initial certificate on file — the CoQ keeps its planned number with a provisional date 27.05.2026 | P060332: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-6-K-26 of 07.08.2026 / 197-6-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060352: no initial certificate on file — the CoQ keeps its planned number with a provisional date 28.05.2026 | P060352: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-7-K-26 of 07.08.2026 / 197-7-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060382: no initial certificate on file — the CoQ keeps its planned number with a provisional date 01.06.2026 | P060382: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-21-K-26 of 07.08.2026 / 197-21-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060282: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060162: no initial certificate for #9 — only the retest 549-1080-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P050142: no initial certificate for #9 — only the retest 559-1090-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060102: no initial certificate for #9 — only the retest 551-1082-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue)</t>
+          <t>Head of QC, 05.09.2026: preliminary CoQ issuance register — codes CoQ-PP_26-nnn (nnn = 001 … 999), one series for the year of issue, in the order of issue. LEGACY lots (packed before the SOP floor of 11.05.2026, or holding an old in-house QCCoA 001 certificate, which the CoQ supersedes) are all issued on 27.05.2026, in chronological order of packaging; POST-SOP lots follow, each on the first working day 7 days after the latest eCoA the CoQ cites and never before 27.05.2026, so the legacy series keeps 001 onward. Every CoQ cites its lot's iCoA (identification A, B, foreign matter) and reports identification C as 'Conforms', referenced to the eCoA that covers Total THC. ADHERENCE (ISSUE_COQ_CONVENTIONS): a CoQ never precedes a document it cites — a legacy lot whose latest eCoA is dated after 27.05.2026 takes the post-SOP rule and is flagged in Status; a CoQ never precedes its iCoA; Head of QC, 05.09.2026 (evening): a production lot whose initial certificate for a determination is not on file keeps its planned CoQ and number — the initial testing exists at the Faculty of Pharmacy's Center for Natural Products (microbiology: IJZ) and the certificate is to be located (Work Order; Status names the determination); a certificate dated on or after 01.07.2026 is a retest document (the QP's campaign: Tranche 1, the first 21 lots, sampled July 2026; then Tranches 2 and 3) and never certifies the initial CoQ — a determination whose only certificate is a retest one is uncertified for the legacy CoQ and flagged; the IJZ-MB delivery of 25/26.08.2026 (certificates of 31.08 and 01.09.2026, 68 to 436 days after packaging) is one campaign sampling and every certificate in it is a retest document, for the post-SOP lots too; nothing is dated on a weekend. RETEST ROWS: the reissued CoQ carries the retest results (cannabinoids with identification C by Farmahem, mycotoxins, microbiology by IJZ-MB) and the initial certificates for the rest; its rule date is the first working day 7 days after the latest retest certificate, and it is issued once the in-house retest iCoA exists. FORMULAS: No. and the code as on the iCoA Register; Rule date is 27.05.2026 for a legacy row whose latest eCoA is on or before it, else the first working day 7 days after the latest eCoA (not before 27.05.2026); the planned date is the latest of the rule date, the iCoA's date and the lot's last day of packaging; iCoA (register) and its date are looked up on the iCoA Register by Key. The latest eCoA cited is a value (the first credited certificate per determination dated before the retest campaign; for a retest row, the latest retest certificate), recomputed by the builder. Working days are Monday to Friday; public holidays are not applied. FLAGS: P060272: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060322: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060432: no initial certificate for #9 — only the retest 537-1068-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060392: no initial certificate for #9 — only the retest 538-1069-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060292: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060302: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060402: no initial certificate for #10 — only the retest 197-8-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060142: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060182: no initial certificate for #9 — only the retest 550-1081-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | HPA1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-13-K-26 of 07.08.2026 / 197-13-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060152: no initial certificate for #10 — only the retest 197-16-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060202: no initial certificate for #9 — only the retest 547-1078-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060262: post-SOP CoQ rule date 30.04.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060312: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060482: CoQ rule date 07.07.2026 precedes the packaging of the lot (05.08.2026) — held to the packaging date | OPM1024: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-17-K-26 of 07.08.2026 / 197-17-M-26 of 10.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060222: no initial certificate for #9 — only the retest 546-1077-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060332: no initial certificate on file — the CoQ keeps its planned number with a provisional date 27.05.2026 | P060332: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-6-K-26 of 07.08.2026 / 197-6-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060352: no initial certificate on file — the CoQ keeps its planned number with a provisional date 28.05.2026 | P060352: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-7-K-26 of 07.08.2026 / 197-7-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060382: no initial certificate on file — the CoQ keeps its planned number with a provisional date 01.06.2026 | P060382: no initial certificate for #3, #4, #5, #6, #8, #10 — only the retest 197-21-K-26 of 07.08.2026 / 197-21-M-26 of 10.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060442: no initial certificate for #9 — only the retest 536-1067-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060282: post-SOP CoQ rule date 18.05.2026 precedes the legacy series day 27.05.2026 — held to it, so the legacy CoQs keep 001 onward | P060162: no initial certificate for #9 — only the retest 549-1080-26 of 31.08.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P050142: no initial certificate for #9 — only the retest 559-1090-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060102: no initial certificate for #9 — only the retest 551-1082-26 of 01.09.2026; the legacy CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue) | P060342: no initial certificate on file — the CoQ keeps its planned number with a provisional date 01.06.2026 | P060342: no initial certificate for #9 — only the retest 539-1070-26 of 31.08.2026; the post-SOP CoQ cannot cite it (Head of QC to rule: report as not tested at initial testing, or wait for the reissue)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: verify_workbook.py, and the three defects it found in v11
A checker that reads a built workbook as written and recalculated, and
tests every sheet: coverage against the tracker, the dashboard against
coverage, Parameters and row 3 against the desk's criteria, Batch Dates
against the CSV, both registers against their numbering and dating
rules, iCoA Issuance against the registers, and every printed result
against the two-read record of its certificate (5,567 comparisons, none
differing), with the specification verdicts against the criteria.

Fixed what it found: the three P16 lots shared one register key (the key
now accepts any Pnnnnnn, not only P0nnnnn); Batch Coverage and the
tracker used two different placeholders for a lot without a CU code; the
Credit Audit row for the reported non-conformance had no action. v11
passes with no finding.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_gap_analysis/tracker/Issuance_Registers_prelim.xlsx
+++ b/deliverables/qc_gap_analysis/tracker/Issuance_Registers_prelim.xlsx
@@ -7123,7 +7123,7 @@
         </is>
       </c>
       <c r="N81" s="2">
-        <f>IFERROR(INDEX('CoQ Register'!$B:$B,MATCH("— not recorded —|I",'CoQ Register'!$S:$S,0)),"—")</f>
+        <f>IFERROR(INDEX('CoQ Register'!$B:$B,MATCH("P160012|I",'CoQ Register'!$S:$S,0)),"—")</f>
         <v/>
       </c>
       <c r="O81" s="6" t="inlineStr">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="P81" s="2" t="inlineStr">
         <is>
-          <t>— not recorded —|I</t>
+          <t>P160012|I</t>
         </is>
       </c>
       <c r="Q81" s="8" t="inlineStr">
@@ -7200,7 +7200,7 @@
         </is>
       </c>
       <c r="N82" s="2">
-        <f>IFERROR(INDEX('CoQ Register'!$B:$B,MATCH("— not recorded —|I",'CoQ Register'!$S:$S,0)),"—")</f>
+        <f>IFERROR(INDEX('CoQ Register'!$B:$B,MATCH("P160022|I",'CoQ Register'!$S:$S,0)),"—")</f>
         <v/>
       </c>
       <c r="O82" s="6" t="inlineStr">
@@ -7210,7 +7210,7 @@
       </c>
       <c r="P82" s="2" t="inlineStr">
         <is>
-          <t>— not recorded —|I</t>
+          <t>P160022|I</t>
         </is>
       </c>
       <c r="Q82" s="8" t="inlineStr">
@@ -7277,7 +7277,7 @@
         </is>
       </c>
       <c r="N83" s="2">
-        <f>IFERROR(INDEX('CoQ Register'!$B:$B,MATCH("— not recorded —|I",'CoQ Register'!$S:$S,0)),"—")</f>
+        <f>IFERROR(INDEX('CoQ Register'!$B:$B,MATCH("P160032|I",'CoQ Register'!$S:$S,0)),"—")</f>
         <v/>
       </c>
       <c r="O83" s="6" t="inlineStr">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="P83" s="2" t="inlineStr">
         <is>
-          <t>— not recorded —|I</t>
+          <t>P160032|I</t>
         </is>
       </c>
       <c r="Q83" s="8" t="inlineStr">
@@ -21129,11 +21129,11 @@
         </is>
       </c>
       <c r="H82" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("— not recorded —|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P160012|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I82" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("— not recorded —|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P160012|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -21179,7 +21179,7 @@
       </c>
       <c r="S82" s="2" t="inlineStr">
         <is>
-          <t>— not recorded —|I</t>
+          <t>P160012|I</t>
         </is>
       </c>
       <c r="T82" s="9" t="inlineStr">
@@ -21219,11 +21219,11 @@
         </is>
       </c>
       <c r="H83" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("— not recorded —|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P160022|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I83" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("— not recorded —|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P160022|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -21269,7 +21269,7 @@
       </c>
       <c r="S83" s="2" t="inlineStr">
         <is>
-          <t>— not recorded —|I</t>
+          <t>P160022|I</t>
         </is>
       </c>
       <c r="T83" s="9" t="inlineStr">
@@ -21309,11 +21309,11 @@
         </is>
       </c>
       <c r="H84" s="2">
-        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("— not recorded —|I",'iCoA Register'!$P:$P,0)),"—")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$B:$B,MATCH("P160032|I",'iCoA Register'!$P:$P,0)),"—")</f>
         <v/>
       </c>
       <c r="I84" s="5">
-        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("— not recorded —|I",'iCoA Register'!$P:$P,0)),"")</f>
+        <f>IFERROR(INDEX('iCoA Register'!$D:$D,MATCH("P160032|I",'iCoA Register'!$P:$P,0)),"")</f>
         <v/>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -21359,7 +21359,7 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
-          <t>— not recorded —|I</t>
+          <t>P160032|I</t>
         </is>
       </c>
       <c r="T84" s="9" t="inlineStr">

</xml_diff>